<commit_message>
Correct Pons recovery reserve to quote fees
</commit_message>
<xml_diff>
--- a/excel/latest/PonsV2_股票Quote控筹模型.xlsx
+++ b/excel/latest/PonsV2_股票Quote控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="R1503447c5fe24ac7"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R121b487aa5444b30"/>
+    <sheet name="控筹模型" sheetId="1" r:id="Rf7e4b787ee604d02"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R4dbb6c88067644a8"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1531,7 +1531,7 @@
         <v>恢复目标控筹预留</v>
       </c>
       <c r="D26" s="122">
-        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",IF(AND($J$55&gt;0,$J$56&gt;0),MAX(0,$G$50/$J$55-$G$50/$J$56),""))</f>
+        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",0)</f>
       </c>
       <c r="E26" s="106">
         <f>$D$7</f>
@@ -1700,7 +1700,7 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="115" t="str">
-        <v>Pons 外盘买入时 Hook fee 与 Creator Tax 从输出 Meme 扣除，卖出时从输出 Quote 扣除。洗筹后 Meme 持仓会按买入侧费率减少；补回按洗后 TOKEN 缺口与现有 V4 曲线差额估算，不重复计入洗筹损耗。</v>
+        <v>Pons V2 外盘手续费始终按 Quote leg 计收；Hook 某些方向暂存的 Meme 费用会在池内转换回 Quote，属于内部归集路径。按本模型口径不降低 TOKEN 控筹率，因此恢复目标控筹预留为 0。</v>
       </c>
       <c r="D36" s="115"/>
       <c r="E36" s="115"/>
@@ -2121,7 +2121,7 @@
         <v>洗后持仓保留比例</v>
       </c>
       <c r="J54" s="112">
-        <f>MAX(0,1-$G$42-$J$7)</f>
+        <f>1</f>
       </c>
       <c r="K54" s="107"/>
       <c r="L54" s="107"/>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="I6" s="153"/>
       <c r="J6" s="153" t="str">
-        <v>V4 Hook 按交易方向从输出币收取；买入输出为 Meme，卖出输出为 Quote。</v>
+        <v>费用始终按 Quote leg 计收；Hook 暂存的 Meme 费用会转换回 Quote。</v>
       </c>
       <c r="K6" s="153"/>
       <c r="L6" s="153"/>

</xml_diff>

<commit_message>
Add Pons USDG quote to Excel downloads
</commit_message>
<xml_diff>
--- a/excel/latest/PonsV2_股票Quote控筹模型.xlsx
+++ b/excel/latest/PonsV2_股票Quote控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="R4da12d0f94ab4c51"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R82fe03f62c564d75"/>
+    <sheet name="控筹模型" sheetId="1" r:id="R6c70b30a17644365"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R3ed7d1eb6cff4109"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -164,7 +164,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="155">
+  <x:cellXfs count="158">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -621,6 +621,11 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1123,7 +1128,7 @@
         <v>Quote</v>
       </c>
       <c r="D7" s="51" t="str">
-        <v>ETH</v>
+        <v>USDG</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="35" t="str">
@@ -1393,7 +1398,7 @@
         <v>原生币价格 / USDT</v>
       </c>
       <c r="J19" s="123">
-        <f>IF($D$7="ETH",$D$55,IF(VLOOKUP("ETH",'Quote参数'!$E$9:$S$62,15,FALSE)&gt;0,VLOOKUP("ETH",'Quote参数'!$E$9:$S$62,15,FALSE),""))</f>
+        <f>IF($D$7="ETH",$D$55,IF(VLOOKUP("ETH",'Quote参数'!$E$9:$S$63,15,FALSE)&gt;0,VLOOKUP("ETH",'Quote参数'!$E$9:$S$63,15,FALSE),""))</f>
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="106"/>
@@ -1789,7 +1794,7 @@
         <v>Quote 名称</v>
       </c>
       <c r="D41" s="108">
-        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$62,2,FALSE)</f>
+        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$63,2,FALSE)</f>
       </c>
       <c r="E41" s="107"/>
       <c r="F41" s="107" t="str">
@@ -1815,7 +1820,7 @@
         <v>Quote 合约</v>
       </c>
       <c r="D42" s="109">
-        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$62,3,FALSE)</f>
+        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$63,3,FALSE)</f>
       </c>
       <c r="E42" s="107"/>
       <c r="F42" s="107" t="str">
@@ -1863,14 +1868,14 @@
         <v>Decimals</v>
       </c>
       <c r="D44" s="110">
-        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$62,4,FALSE)</f>
+        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$63,4,FALSE)</f>
       </c>
       <c r="E44" s="107"/>
       <c r="F44" s="107" t="str">
         <v>毕业真实 Quote</v>
       </c>
       <c r="G44" s="108">
-        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$62,6,FALSE)</f>
+        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$63,6,FALSE)</f>
       </c>
       <c r="H44" s="107"/>
       <c r="I44" s="107" t="str">
@@ -1915,14 +1920,14 @@
         <v>协议参数证据</v>
       </c>
       <c r="D46" s="108">
-        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$P$62,12,FALSE)</f>
+        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$P$63,12,FALSE)</f>
       </c>
       <c r="E46" s="107"/>
       <c r="F46" s="107" t="str">
         <v>phantom Quote</v>
       </c>
       <c r="G46" s="108">
-        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$62,5,FALSE)</f>
+        <f>VLOOKUP($D$7,'Quote参数'!$E$9:$J$63,5,FALSE)</f>
       </c>
       <c r="H46" s="107"/>
       <c r="I46" s="107" t="str">
@@ -2133,7 +2138,7 @@
         <v>Quote 价格 / USDT</v>
       </c>
       <c r="D55" s="108">
-        <f>IF($D$9&lt;&gt;"",IF(AND(ISNUMBER($D$9),$D$9&gt;0),$D$9,""),IF(VLOOKUP($D$7,'Quote参数'!$E$9:$S$62,15,FALSE)&gt;0,VLOOKUP($D$7,'Quote参数'!$E$9:$S$62,15,FALSE),""))</f>
+        <f>IF($D$9&lt;&gt;"",IF(AND(ISNUMBER($D$9),$D$9&gt;0),$D$9,""),IF(VLOOKUP($D$7,'Quote参数'!$E$9:$S$63,15,FALSE)&gt;0,VLOOKUP($D$7,'Quote参数'!$E$9:$S$63,15,FALSE),""))</f>
       </c>
       <c r="E55" s="107"/>
       <c r="F55" s="107" t="str">
@@ -2159,7 +2164,7 @@
         <v>行情时间 / UTC</v>
       </c>
       <c r="D56" s="150">
-        <f>IF(VLOOKUP($D$7,'Quote参数'!$E$9:$T$62,16,FALSE)=0,"",VLOOKUP($D$7,'Quote参数'!$E$9:$T$62,16,FALSE))</f>
+        <f>IF(VLOOKUP($D$7,'Quote参数'!$E$9:$T$63,16,FALSE)=0,"",VLOOKUP($D$7,'Quote参数'!$E$9:$T$63,16,FALSE))</f>
       </c>
       <c r="E56" s="107"/>
       <c r="F56" s="107" t="str">
@@ -4284,7 +4289,7 @@
   </conditionalFormatting>
   <dataValidations count="13">
     <dataValidation type="list" sqref="D7">
-      <formula1>'Quote参数'!$E$9:$E$62</formula1>
+      <formula1>'Quote参数'!$E$9:$E$63</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="between" sqref="D8">
       <formula1>0</formula1>
@@ -4414,7 +4419,7 @@
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="6" t="str">
-        <v>ETH + 53 个股票 / ETF Quote。股票类参数为 Robinhood Chain 区块 54,430,299 快照；Factory owner 后续可更新新 Launch 参数。</v>
+        <v>ETH、USDG 与股票 / ETF Quote。USDG 参数取 Factory 区块 68,708,148；已发币以发行时快照为准。</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -4549,9 +4554,11 @@
       <c r="F7" s="35"/>
       <c r="G7" s="35"/>
       <c r="H7" s="35" t="str">
-        <v>Snipe 窗口</v>
-      </c>
-      <c r="I7" s="35"/>
+        <v>USDG 参数依据</v>
+      </c>
+      <c r="I7" s="35" t="str">
+        <v>https://robinhoodchain.blockscout.com/address/0x7eD598BcEf8bd9Edd8C97A195C6d13f40801EC7e?tab=read_contract</v>
+      </c>
       <c r="J7" s="35" t="str">
         <v>3 秒（当前 Factory 链上参数）</v>
       </c>
@@ -8367,6 +8374,72 @@
       <c r="V62" s="34" t="inlineStr">
         <is>
           <t>暂无合格池价；可手动输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="42" customHeight="1">
+      <c r="C63" t="n">
+        <v>55</v>
+      </c>
+      <c r="D63" t="str">
+        <v>稳定币</v>
+      </c>
+      <c r="E63" t="str">
+        <v>USDG</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Global Dollar</v>
+      </c>
+      <c r="G63" t="str">
+        <v>​0x5fc5360D0400a0Fd4f2af552ADD042D716F1d168</v>
+      </c>
+      <c r="H63" t="n">
+        <v>6</v>
+      </c>
+      <c r="I63" t="n">
+        <v>202.25</v>
+      </c>
+      <c r="J63" t="n">
+        <v>505.625</v>
+      </c>
+      <c r="K63">
+        <f>J63/I63</f>
+      </c>
+      <c r="L63">
+        <f>J63</f>
+      </c>
+      <c r="M63">
+        <f>1000000000*I63*J63/(I63+J63)^2</f>
+      </c>
+      <c r="N63">
+        <f>1000000000*I63^2/(I63+J63)^2</f>
+      </c>
+      <c r="O63">
+        <f>1-N63/1000000000</f>
+      </c>
+      <c r="P63" t="n">
+        <v>68708148</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Approved / ERC-20</v>
+      </c>
+      <c r="R63" t="str">
+        <v>https://robinhoodchain.blockscout.com/address/0x5fc5360d0400a0fd4f2af552add042d716f1d168</v>
+      </c>
+      <c r="S63" s="155">
+        <v>1.0003961568781237</v>
+      </c>
+      <c r="T63" s="156">
+        <v>46285.27349457176</v>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>https://api.coingecko.com/api/v3/simple/price?ids=tether&amp;vs_currencies=usd</t>
+        </is>
+      </c>
+      <c r="V63" s="157" t="inlineStr">
+        <is>
+          <t>USDG 按 1 USD 估算；本地可手动更新</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Pons USDG launch snapshot to 8090
</commit_message>
<xml_diff>
--- a/excel/latest/PonsV2_股票Quote控筹模型.xlsx
+++ b/excel/latest/PonsV2_股票Quote控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="控筹模型" sheetId="1" r:id="R6c70b30a17644365"/>
-    <sheet name="Quote参数" sheetId="2" r:id="R3ed7d1eb6cff4109"/>
+    <sheet name="控筹模型" sheetId="1" r:id="Rd7aedc8ed7d34244"/>
+    <sheet name="Quote参数" sheetId="2" r:id="R2337eec321c940d1"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -4419,7 +4419,7 @@
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="6" t="str">
-        <v>ETH、USDG 与股票 / ETF Quote。USDG 参数取 Factory 区块 68,708,148；已发币以发行时快照为准。</v>
+        <v>ETH、USDG 与股票 / ETF Quote。USDG 采用 TRAIN 发行参数快照，外盘 8,090 USDG；新币参数可变。</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
@@ -4557,7 +4557,7 @@
         <v>USDG 参数依据</v>
       </c>
       <c r="I7" s="35" t="str">
-        <v>https://robinhoodchain.blockscout.com/address/0x7eD598BcEf8bd9Edd8C97A195C6d13f40801EC7e?tab=read_contract</v>
+        <v>https://robin.etherscan.io/tx/0x387e3237904e4822075066331564561c373b691fd47ad2d52b4f64fb4f398c84#eventlog</v>
       </c>
       <c r="J7" s="35" t="str">
         <v>3 秒（当前 Factory 链上参数）</v>
@@ -8397,10 +8397,10 @@
         <v>6</v>
       </c>
       <c r="I63" t="n">
-        <v>202.25</v>
+        <v>3236</v>
       </c>
       <c r="J63" t="n">
-        <v>505.625</v>
+        <v>8090</v>
       </c>
       <c r="K63">
         <f>J63/I63</f>
@@ -8418,10 +8418,10 @@
         <f>1-N63/1000000000</f>
       </c>
       <c r="P63" t="n">
-        <v>68708148</v>
+        <v>69045064</v>
       </c>
       <c r="Q63" t="str">
-        <v>Approved / ERC-20</v>
+        <v>已发行实例 / ERC-20</v>
       </c>
       <c r="R63" t="str">
         <v>https://robinhoodchain.blockscout.com/address/0x5fc5360d0400a0fd4f2af552add042d716f1d168</v>

</xml_diff>